<commit_message>
Ajuste de pacotes e caminhos
</commit_message>
<xml_diff>
--- a/analise_agentes.xlsx
+++ b/analise_agentes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B273"/>
+  <dimension ref="A1:B260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,7 +435,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>48481</v>
+        <v>7607</v>
       </c>
     </row>
     <row r="3">
@@ -445,7 +445,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>35871</v>
+        <v>5709</v>
       </c>
     </row>
     <row r="4">
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>31518</v>
+        <v>5043</v>
       </c>
     </row>
     <row r="5">
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>31447</v>
+        <v>4897</v>
       </c>
     </row>
     <row r="6">
@@ -475,27 +475,27 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28764</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Agente do Acidente, </t>
+          <t xml:space="preserve">Metal - Inclui Liga </t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>27152</v>
+        <v>4258</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metal - Inclui Liga </t>
+          <t xml:space="preserve">Agente do Acidente, </t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>27063</v>
+        <v>4206</v>
       </c>
     </row>
     <row r="9">
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>19060</v>
+        <v>3024</v>
       </c>
     </row>
     <row r="10">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16805</v>
+        <v>2696</v>
       </c>
     </row>
     <row r="11">
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15509</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="12">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>13963</v>
+        <v>2175</v>
       </c>
     </row>
     <row r="13">
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>13167</v>
+        <v>2121</v>
       </c>
     </row>
     <row r="14">
@@ -555,27 +555,27 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>11497</v>
+        <v>1916</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Agente Infeccioso ou</t>
+          <t>Escada Movel ou Fixa</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11335</v>
+        <v>1864</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Escada Movel ou Fixa</t>
+          <t>Agente Infeccioso ou</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>11209</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="17">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>10215</v>
+        <v>1571</v>
       </c>
     </row>
     <row r="18">
@@ -595,27 +595,27 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>9973</v>
+        <v>1481</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ferramenta, Maquina,</t>
+          <t xml:space="preserve">Ser Vivo, Nic       </t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>9632</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ser Vivo, Nic       </t>
+          <t>Ferramenta, Maquina,</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>9321</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="21">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>8852</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="22">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>7397</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="23">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6764</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="24">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>6304</v>
+        <v>992</v>
       </c>
     </row>
     <row r="25">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>6108</v>
+        <v>930</v>
       </c>
     </row>
     <row r="26">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>5393</v>
+        <v>879</v>
       </c>
     </row>
     <row r="27">
@@ -685,57 +685,57 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>5294</v>
+        <v>846</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bicicleta           </t>
+          <t xml:space="preserve">Serra - Maquina     </t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>4624</v>
+        <v>766</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Serra - Maquina     </t>
+          <t>Piso de Veiculo - Su</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4608</v>
+        <v>741</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Piso de Veiculo - Su</t>
+          <t xml:space="preserve">Bicicleta           </t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4572</v>
+        <v>733</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Martelo, Malho, Marr</t>
+          <t>Agua - Usar Quando O</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3895</v>
+        <v>614</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Agua - Usar Quando O</t>
+          <t>Martelo, Malho, Marr</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3709</v>
+        <v>600</v>
       </c>
     </row>
     <row r="33">
@@ -745,37 +745,37 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3300</v>
+        <v>548</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Empilhadeira        </t>
+          <t xml:space="preserve">Prensa - Maquina    </t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>3229</v>
+        <v>532</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cadeira Banco - Mobi</t>
+          <t xml:space="preserve">Empilhadeira        </t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>3149</v>
+        <v>519</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prensa - Maquina    </t>
+          <t>Cadeira Banco - Mobi</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>3047</v>
+        <v>502</v>
       </c>
     </row>
     <row r="37">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3045</v>
+        <v>484</v>
       </c>
     </row>
     <row r="38">
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2669</v>
+        <v>427</v>
       </c>
     </row>
     <row r="39">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2660</v>
+        <v>418</v>
       </c>
     </row>
     <row r="40">
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2545</v>
+        <v>385</v>
       </c>
     </row>
     <row r="41">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2409</v>
+        <v>366</v>
       </c>
     </row>
     <row r="42">
@@ -835,47 +835,47 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2330</v>
+        <v>360</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Andaime, Plataforma </t>
+          <t>Particulas - nao Ide</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2190</v>
+        <v>358</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Embalagem e Recipien</t>
+          <t xml:space="preserve">Andaime, Plataforma </t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2169</v>
+        <v>353</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Politriz, Lixadora, </t>
+          <t>Embalagem e Recipien</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2093</v>
+        <v>329</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Particulas - nao Ide</t>
+          <t xml:space="preserve">Politriz, Lixadora, </t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2091</v>
+        <v>325</v>
       </c>
     </row>
     <row r="47">
@@ -885,27 +885,27 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1972</v>
+        <v>313</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Furadeira, Broqueade</t>
+          <t xml:space="preserve">Ataque de Ser Vivo, </t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1908</v>
+        <v>292</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ataque de Ser Vivo, </t>
+          <t>Forno, Estufa, Retor</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1844</v>
+        <v>284</v>
       </c>
     </row>
     <row r="50">
@@ -915,77 +915,77 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1760</v>
+        <v>284</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Corda, Cabo, Corrent</t>
+          <t>Furadeira, Broqueade</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1716</v>
+        <v>279</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Puncao, Ponteiro, Va</t>
+          <t xml:space="preserve">Edificio - Edificio </t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1685</v>
+        <v>278</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Produto Mineral nao </t>
+          <t>Corda, Cabo, Corrent</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1667</v>
+        <v>267</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edificio - Edificio </t>
+          <t xml:space="preserve">Produto Mineral nao </t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1659</v>
+        <v>265</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Serra- Ferramenta Po</t>
+          <t xml:space="preserve">Maquina Agricola    </t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1639</v>
+        <v>247</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maquina Agricola    </t>
+          <t>Tubo Sob Pressao (Ma</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1630</v>
+        <v>245</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Forno, Estufa, Retor</t>
+          <t>Balcao, Bancada - Mo</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1618</v>
+        <v>242</v>
       </c>
     </row>
     <row r="58">
@@ -995,37 +995,37 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1566</v>
+        <v>230</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Balcao, Bancada - Mo</t>
+          <t>Puncao, Ponteiro, Va</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1562</v>
+        <v>229</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Tubo Sob Pressao (Ma</t>
+          <t>Barril, Barrica, Bar</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1502</v>
+        <v>228</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Equip. Eletrico, Nic</t>
+          <t>Serra- Ferramenta Po</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1450</v>
+        <v>223</v>
       </c>
     </row>
     <row r="62">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1429</v>
+        <v>219</v>
       </c>
     </row>
     <row r="63">
@@ -1045,37 +1045,37 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1413</v>
+        <v>216</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Frasco, Garrafa - Em</t>
+          <t>Transportador com Fo</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1347</v>
+        <v>208</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Mesa, Carteira, Exce</t>
+          <t>Frasco, Garrafa - Em</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1325</v>
+        <v>207</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Transportador com Fo</t>
+          <t>Vegetal - Planta, Ar</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1275</v>
+        <v>204</v>
       </c>
     </row>
     <row r="67">
@@ -1085,37 +1085,37 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1260</v>
+        <v>201</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Barril, Barrica, Bar</t>
+          <t>Equip. Eletrico, Nic</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>1253</v>
+        <v>192</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Maquina de Embalar o</t>
+          <t>Mesa, Carteira, Exce</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1242</v>
+        <v>188</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Vegetal - Planta, Ar</t>
+          <t>Maquina de Embalar o</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1155</v>
+        <v>188</v>
       </c>
     </row>
     <row r="71">
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>1151</v>
+        <v>175</v>
       </c>
     </row>
     <row r="72">
@@ -1135,177 +1135,177 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1121</v>
+        <v>172</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Produto de Limpeza, </t>
+          <t>Alavanca, Pe-De-Cabr</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1116</v>
+        <v>172</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Alavanca, Pe-De-Cabr</t>
+          <t>Edificio ou Estrutur</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1107</v>
+        <v>171</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Laminadora, Calandra</t>
+          <t>Sucata, Entulho, Res</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1054</v>
+        <v>171</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Tesoura, Tesourao- F</t>
+          <t>Laminadora, Calandra</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1049</v>
+        <v>168</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ferramenta Portatil </t>
+          <t>Esforco Excessivo ao</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>1031</v>
+        <v>164</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Edificio ou Estrutur</t>
+          <t>Misturador, Batedeir</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>1023</v>
+        <v>157</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Reacao do Corpo a Mo</t>
+          <t>Plastico - Inclui Po</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>1001</v>
+        <v>154</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Sucata, Entulho, Res</t>
+          <t>Reacao do Corpo a Mo</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>991</v>
+        <v>154</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Misturador, Batedeir</t>
+          <t>Tesoura, Tesourao- F</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>976</v>
+        <v>152</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Esforco Excessivo ao</t>
+          <t xml:space="preserve">Ferramenta Portatil </t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>951</v>
+        <v>151</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Serra, Serrote- Ferr</t>
+          <t>Tijolo e Telha - Cer</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>941</v>
+        <v>144</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Chave de Parafuso- F</t>
+          <t xml:space="preserve">Maquina de Costurar </t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>913</v>
+        <v>144</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maquina de Costurar </t>
+          <t xml:space="preserve">Acido               </t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>870</v>
+        <v>141</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Plastico - Inclui Po</t>
+          <t>Serra, Serrote- Ferr</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>815</v>
+        <v>138</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Esmeril- Ferramenta </t>
+          <t>Chave de Parafuso- F</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>811</v>
+        <v>134</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Corrente, Corda, Cab</t>
+          <t xml:space="preserve">Esmeril- Ferramenta </t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>782</v>
+        <v>133</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Tubo, Manilha - Cera</t>
+          <t xml:space="preserve">Produto de Limpeza, </t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>780</v>
+        <v>130</v>
       </c>
     </row>
     <row r="90">
@@ -1315,27 +1315,27 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>779</v>
+        <v>126</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Tijolo e Telha - Cer</t>
+          <t>Tubo, Manilha - Cera</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>772</v>
+        <v>122</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Cortadeira, Guilhoti</t>
+          <t>Elevador - Equip. de</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>766</v>
+        <v>120</v>
       </c>
     </row>
     <row r="93">
@@ -1345,97 +1345,97 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>721</v>
+        <v>118</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Tambor, Polia, Rolda</t>
+          <t>Corrente, Corda, Cab</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>709</v>
+        <v>117</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trator              </t>
+          <t>Correia - Dispositiv</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>681</v>
+        <v>116</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Elevador - Equip. de</t>
+          <t xml:space="preserve">Area ou Ambiente de </t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>659</v>
+        <v>113</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Arquivo, Fichario, E</t>
+          <t>Cortadeira, Guilhoti</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>651</v>
+        <v>112</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Area ou Ambiente de </t>
+          <t>Arquivo, Fichario, E</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>641</v>
+        <v>99</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Deposito Fixo (Tanqu</t>
+          <t>Tambor, Polia, Rolda</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>641</v>
+        <v>97</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Correia - Dispositiv</t>
+          <t xml:space="preserve">Ceramica            </t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>631</v>
+        <v>96</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Equip. de Guindar, N</t>
+          <t>Maquina de Aparafusa</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>626</v>
+        <v>94</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Ferramenta de Soldag</t>
+          <t xml:space="preserve">Trator              </t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>626</v>
+        <v>93</v>
       </c>
     </row>
     <row r="103">
@@ -1445,407 +1445,407 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>617</v>
+        <v>91</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Acido               </t>
+          <t>Ferramenta de Soldag</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>611</v>
+        <v>90</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Maquina de Aparafusa</t>
+          <t>Composto Metalico (D</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>583</v>
+        <v>88</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Composto Metalico (D</t>
+          <t>Motor Eletrico - Equ</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>568</v>
+        <v>87</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ceramica            </t>
+          <t>Deposito Fixo (Tanqu</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>551</v>
+        <v>85</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Maquina de Fundir, d</t>
+          <t>Chave de Porca ou de</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>532</v>
+        <v>82</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Alicate, Torques, Te</t>
+          <t>Macaco (Mecanico, Hi</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>530</v>
+        <v>78</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Vaso Sob Pressao (Pa</t>
+          <t>Equip. de Guindar, N</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>507</v>
+        <v>77</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Motor, Bomba, Turbin</t>
+          <t>Maquina de Fundir, d</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>497</v>
+        <v>76</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Chave de Porca ou de</t>
+          <t>Motor, Bomba, Turbin</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>486</v>
+        <v>73</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Macaco (Mecanico, Hi</t>
+          <t>Cais, Doca - Edifici</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>480</v>
+        <v>68</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Motor Eletrico - Equ</t>
+          <t>Vaso Sob Pressao (Pa</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>479</v>
+        <v>67</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Queda de Pes. com Di</t>
+          <t xml:space="preserve">Produto Animal, Nic </t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>413</v>
+        <v>66</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Ponte Rolante - Equi</t>
+          <t>Alicate, Torques, Te</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>409</v>
+        <v>66</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Produto Alimenticio </t>
+          <t>Ponte Rolante - Equi</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>404</v>
+        <v>64</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Energia             </t>
+          <t>Queda de Pes. com Di</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>393</v>
+        <v>63</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Cais, Doca - Edifici</t>
+          <t>Maquina de Terraplen</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>392</v>
+        <v>62</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Britador, Moinho - M</t>
+          <t xml:space="preserve">Carne e Derivados - </t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>382</v>
+        <v>62</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Produtos Alimenticio</t>
+          <t>Plaina, Tupia - Maqu</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>381</v>
+        <v>61</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Maquina de Terraplen</t>
+          <t xml:space="preserve">Tapete, Forracao de </t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>378</v>
+        <v>58</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oleo Combustivel    </t>
+          <t>Guindaste - Equip. d</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>372</v>
+        <v>58</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Martelete, Socador- </t>
+          <t>Escavacao (Para Edif</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>371</v>
+        <v>58</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impacto Sofrido por </t>
+          <t>Impacto de Pes. Cont</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>359</v>
+        <v>57</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Engrenagem - Disposi</t>
+          <t>Britador, Moinho - M</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>354</v>
+        <v>57</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Produto Animal, Nic </t>
+          <t xml:space="preserve">Painel de Controle, </t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>353</v>
+        <v>55</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carne e Derivados - </t>
+          <t xml:space="preserve">Oleo Combustivel    </t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>350</v>
+        <v>55</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Painel de Controle, </t>
+          <t>Veiculo Sobre Trilho</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>339</v>
+        <v>54</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tapete, Forracao de </t>
+          <t>Condutor - Equip. El</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>339</v>
+        <v>53</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Condutor - Equip. El</t>
+          <t xml:space="preserve">Produto Alimenticio </t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>338</v>
+        <v>53</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Impacto de Pes. Cont</t>
+          <t xml:space="preserve">Ceramica, Nic       </t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>318</v>
+        <v>51</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Dispositivo de Trans</t>
+          <t xml:space="preserve">Energia             </t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>315</v>
+        <v>51</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Poco, Entrada, Galer</t>
+          <t>Dispositivo de Trans</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>311</v>
+        <v>50</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Plaina, Tupia - Maqu</t>
+          <t>Revestimento Ceramic</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>310</v>
+        <v>50</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Masarico - Ferrament</t>
+          <t>Produtos Alimenticio</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>308</v>
+        <v>49</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Veiculo Sobre Trilho</t>
+          <t xml:space="preserve">Martelete, Socador- </t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>307</v>
+        <v>48</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Guindaste - Equip. d</t>
+          <t xml:space="preserve">Caldeira            </t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>303</v>
+        <v>48</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Talha - Equip. de Gu</t>
+          <t xml:space="preserve">Canal, Fosso        </t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>290</v>
+        <v>48</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ceramica, Nic       </t>
+          <t>Poco, Entrada, Galer</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>286</v>
+        <v>47</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Revestimento Ceramic</t>
+          <t xml:space="preserve">Maquina de Imprimir </t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>285</v>
+        <v>47</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Canal, Fosso        </t>
+          <t xml:space="preserve">Bomba               </t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>285</v>
+        <v>45</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Texteis - Inclui Fib</t>
+          <t>Talha - Equip. de Gu</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>285</v>
+        <v>44</v>
       </c>
     </row>
     <row r="144">
@@ -1855,87 +1855,87 @@
         </is>
       </c>
       <c r="B144" t="n">
-        <v>285</v>
+        <v>44</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Equip. de Aqueciment</t>
+          <t>Engrenagem - Disposi</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>279</v>
+        <v>43</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vestuario, Nic      </t>
+          <t>Masarico - Ferrament</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>276</v>
+        <v>42</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maquina de Imprimir </t>
+          <t>Perfuratriz- Ferrame</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>273</v>
+        <v>42</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caldeira            </t>
+          <t xml:space="preserve">Vestuario, Nic      </t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>273</v>
+        <v>42</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Escavacao (Para Edif</t>
+          <t>Papel e Pasta para P</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>259</v>
+        <v>42</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Escavacao, Fosso, Tu</t>
+          <t>Texteis - Inclui Fib</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>250</v>
+        <v>40</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Louca Sanitaria (Pia</t>
+          <t xml:space="preserve">Impacto Sofrido por </t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>248</v>
+        <v>39</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Pa, Cavadeira- Ferra</t>
+          <t>Osso - Produto Anima</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>247</v>
+        <v>36</v>
       </c>
     </row>
     <row r="153">
@@ -1945,77 +1945,77 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>246</v>
+        <v>35</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Papel e Pasta para P</t>
+          <t>Ponte, Viaduto - Edi</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>244</v>
+        <v>35</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Perfuratriz- Ferrame</t>
+          <t>Medicamento em Geral</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>237</v>
+        <v>34</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Osso - Produto Anima</t>
+          <t>Equip. de Aqueciment</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>230</v>
+        <v>34</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Piso de Mina - Super</t>
+          <t>Louca Sanitaria (Pia</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>229</v>
+        <v>33</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Medicamento em Geral</t>
+          <t>Pa, Cavadeira- Ferra</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>210</v>
+        <v>32</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ruido               </t>
+          <t>Escavacao, Fosso, Tu</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>200</v>
+        <v>32</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Veiculo de Terraplen</t>
+          <t>Piso de Mina - Super</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>197</v>
+        <v>31</v>
       </c>
     </row>
     <row r="161">
@@ -2025,1126 +2025,996 @@
         </is>
       </c>
       <c r="B161" t="n">
-        <v>194</v>
+        <v>31</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bomba               </t>
+          <t>Reostato, Dispositiv</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>189</v>
+        <v>30</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Transportador por Gr</t>
+          <t>Parafina, Oleo Lubri</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>179</v>
+        <v>30</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Parafina, Oleo Lubri</t>
+          <t>Lima, Grosa- Ferrame</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>166</v>
+        <v>29</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aerodispersoides    </t>
+          <t>Enxada, Enxadao, Sac</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>159</v>
+        <v>29</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Peneira Mecanica, Ma</t>
+          <t>Produto Mineral Meta</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>156</v>
+        <v>28</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Ponte, Viaduto - Edi</t>
+          <t>Formao, Cinzel- Ferr</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>156</v>
+        <v>28</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Atrito ou Abrasao po</t>
+          <t>Garfo, Ancinho, Forc</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>156</v>
+        <v>26</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Luminaria, Globo, Ia</t>
+          <t>Veiculo de Terraplen</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>152</v>
+        <v>26</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Enxada, Enxadao, Sac</t>
+          <t xml:space="preserve">Ruido               </t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>147</v>
+        <v>25</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arco Eletrico       </t>
+          <t>Atrito ou Abrasao po</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>146</v>
+        <v>25</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Produto Mineral Meta</t>
+          <t>Maquina de Mineracao</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>145</v>
+        <v>24</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alcool              </t>
+          <t xml:space="preserve">Arco Eletrico       </t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>145</v>
+        <v>23</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Politriz, Enceradeir</t>
+          <t>Peneira Mecanica, Ma</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>137</v>
+        <v>22</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t xml:space="preserve">Equip. Eletrolitico </t>
+          <t>Gas Carbonico (Dioxi</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>135</v>
+        <v>22</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Garfo, Ancinho, Forc</t>
+          <t xml:space="preserve">Equip. Eletrolitico </t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>130</v>
+        <v>22</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fruta e Derivados   </t>
+          <t>Transportador por Gr</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>126</v>
+        <v>22</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Maquina de Mineracao</t>
+          <t xml:space="preserve">Aeronave            </t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>123</v>
+        <v>21</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Pua, Trado, Verruma,</t>
+          <t>Pressao Ambiente, Ex</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>123</v>
+        <v>21</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Reostato, Dispositiv</t>
+          <t xml:space="preserve">Exposicao a Pressao </t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>122</v>
+        <v>21</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Formao, Cinzel- Ferr</t>
+          <t>Luminaria, Globo, Ia</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>120</v>
+        <v>21</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Pressao Ambiente, Ex</t>
+          <t>Pua, Trado, Verruma,</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>111</v>
+        <v>21</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Lima, Grosa- Ferrame</t>
+          <t>Temperatura Ambiente</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>110</v>
+        <v>20</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Equip. para Trabalho</t>
+          <t>Rebitadeira- Ferrame</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>110</v>
+        <v>18</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aeronave            </t>
+          <t>Politriz, Enceradeir</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>108</v>
+        <v>18</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rebocador Mecanico, </t>
+          <t>Transformador, Conve</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>106</v>
+        <v>17</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exposicao a Pressao </t>
+          <t xml:space="preserve">Alcool              </t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>104</v>
+        <v>17</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Temperatura Ambiente</t>
+          <t>Guincho Eletrico - E</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>101</v>
+        <v>17</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Transformador, Conve</t>
+          <t>Veiculo de Tracao An</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>100</v>
+        <v>16</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Picareta- Ferramenta</t>
+          <t>Caldeira, Vaso Sob P</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>99</v>
+        <v>15</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Rebitadeira- Ferrame</t>
+          <t>Gasolina (Exceto Qua</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>95</v>
+        <v>15</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Gasoleo, Oleo Diesel</t>
+          <t>Equip. de Iluminacao</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>92</v>
+        <v>14</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Gasolina (Exceto Qua</t>
+          <t>Guincho Pneumatico -</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>91</v>
+        <v>14</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Gerador - Equip. Ele</t>
+          <t>Legume, Verdura e De</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>89</v>
+        <v>14</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Guincho Pneumatico -</t>
+          <t xml:space="preserve">Rebocador Mecanico, </t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>86</v>
+        <v>14</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Caldeira, Vaso Sob P</t>
+          <t>Gerador - Equip. Ele</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>86</v>
+        <v>14</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Equip. de Iluminacao</t>
+          <t>Plaina- Ferramenta M</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>85</v>
+        <v>14</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alcali              </t>
+          <t>Equip. para Trabalho</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>84</v>
+        <v>14</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Guincho Eletrico - E</t>
+          <t xml:space="preserve">Cereal e Derivados  </t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>84</v>
+        <v>13</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Leite e Derivados - </t>
+          <t xml:space="preserve">Aerodispersoides    </t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>83</v>
+        <v>12</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Plaina- Ferramenta M</t>
+          <t xml:space="preserve">Triciclo            </t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>82</v>
+        <v>12</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Pa Mecanica, Draga -</t>
+          <t xml:space="preserve">Ferramenta Acionada </t>
         </is>
       </c>
       <c r="B202" t="n">
-        <v>81</v>
+        <v>12</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Veiculo de Tracao An</t>
+          <t>Arco Eletrico - Equi</t>
         </is>
       </c>
       <c r="B203" t="n">
-        <v>80</v>
+        <v>12</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Maquina de Escritori</t>
+          <t>Equip. Emissor de Ra</t>
         </is>
       </c>
       <c r="B204" t="n">
-        <v>78</v>
+        <v>12</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Equip. Emissor de Ra</t>
+          <t>Mesa Elastica Desmon</t>
         </is>
       </c>
       <c r="B205" t="n">
-        <v>77</v>
+        <v>12</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ferramenta Acionada </t>
+          <t xml:space="preserve">Leite e Derivados - </t>
         </is>
       </c>
       <c r="B206" t="n">
-        <v>76</v>
+        <v>11</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Arquibancada, Estadi</t>
+          <t>Machadinha, Enxo- Fe</t>
         </is>
       </c>
       <c r="B207" t="n">
-        <v>76</v>
+        <v>11</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Talhadeira- Ferramen</t>
+          <t xml:space="preserve">Alcali              </t>
         </is>
       </c>
       <c r="B208" t="n">
-        <v>73</v>
+        <v>10</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Arco Eletrico - Equi</t>
+          <t>Talhadeira- Ferramen</t>
         </is>
       </c>
       <c r="B209" t="n">
-        <v>71</v>
+        <v>10</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Legume, Verdura e De</t>
+          <t>Hidrocarboneto Gasos</t>
         </is>
       </c>
       <c r="B210" t="n">
-        <v>69</v>
+        <v>10</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cereal e Derivados  </t>
+          <t>Equip. Magnetico - E</t>
         </is>
       </c>
       <c r="B211" t="n">
-        <v>66</v>
+        <v>10</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Gas Carbonico (Dioxi</t>
+          <t>Composto Organico Ha</t>
         </is>
       </c>
       <c r="B212" t="n">
-        <v>65</v>
+        <v>10</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t xml:space="preserve">Veiculo Aquatico    </t>
+          <t xml:space="preserve">Ruido, Exposicao A  </t>
         </is>
       </c>
       <c r="B213" t="n">
-        <v>64</v>
+        <v>10</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Triciclo            </t>
+          <t xml:space="preserve">Veiculo Aquatico    </t>
         </is>
       </c>
       <c r="B214" t="n">
-        <v>63</v>
+        <v>9</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Hidrocarboneto Gasos</t>
+          <t>Picareta- Ferramenta</t>
         </is>
       </c>
       <c r="B215" t="n">
-        <v>62</v>
+        <v>9</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Machadinha, Enxo- Fe</t>
+          <t>Gasoleo, Oleo Diesel</t>
         </is>
       </c>
       <c r="B216" t="n">
-        <v>59</v>
+        <v>9</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ruido, Exposicao A  </t>
+          <t xml:space="preserve">Neblina             </t>
         </is>
       </c>
       <c r="B217" t="n">
-        <v>57</v>
+        <v>9</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Mesa Elastica Desmon</t>
+          <t xml:space="preserve">Machado- Ferramenta </t>
         </is>
       </c>
       <c r="B218" t="n">
-        <v>57</v>
+        <v>9</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Ataque de Ser Vivo p</t>
+          <t xml:space="preserve">Fruta e Derivados   </t>
         </is>
       </c>
       <c r="B219" t="n">
-        <v>54</v>
+        <v>9</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Neblina             </t>
+          <t>Maquina de Escritori</t>
         </is>
       </c>
       <c r="B220" t="n">
-        <v>49</v>
+        <v>8</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machado- Ferramenta </t>
+          <t>Couro Cru ou Curtido</t>
         </is>
       </c>
       <c r="B221" t="n">
-        <v>48</v>
+        <v>8</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Ferro de Passar- Fer</t>
+          <t xml:space="preserve">Nafta e Solvente de </t>
         </is>
       </c>
       <c r="B222" t="n">
-        <v>46</v>
+        <v>7</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Couro Cru ou Curtido</t>
+          <t>Pa Mecanica, Draga -</t>
         </is>
       </c>
       <c r="B223" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Ataque de Ser Vivo c</t>
+          <t>Ataque de Ser Vivo p</t>
         </is>
       </c>
       <c r="B224" t="n">
-        <v>43</v>
+        <v>7</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Jato de Areia- Ferra</t>
+          <t>Atrito ou Abrasao, N</t>
         </is>
       </c>
       <c r="B225" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Dique, Barragem - Ed</t>
+          <t xml:space="preserve">Equip. de Raios X - </t>
         </is>
       </c>
       <c r="B226" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Equip. Magnetico - E</t>
+          <t>Temperatura Muito Al</t>
         </is>
       </c>
       <c r="B227" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Temperatura Muito Al</t>
+          <t xml:space="preserve">Monoxido de Carbono </t>
         </is>
       </c>
       <c r="B228" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Embreagem de Friccao</t>
+          <t>Jato de Areia- Ferra</t>
         </is>
       </c>
       <c r="B229" t="n">
-        <v>36</v>
+        <v>5</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aprision. Em, Sobre </t>
+          <t xml:space="preserve">Elevador de Cacamba </t>
         </is>
       </c>
       <c r="B230" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nafta e Solvente de </t>
+          <t xml:space="preserve">Tunel               </t>
         </is>
       </c>
       <c r="B231" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Produto de Petroleo </t>
+          <t>Pele, Crina, Pelo, L</t>
         </is>
       </c>
       <c r="B232" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Composto Organico Ha</t>
+          <t>Pau de Carga - Equip</t>
         </is>
       </c>
       <c r="B233" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tunel               </t>
+          <t>Inalacao de Substanc</t>
         </is>
       </c>
       <c r="B234" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Pau de Carga - Equip</t>
+          <t>Ferro de Passar- Fer</t>
         </is>
       </c>
       <c r="B235" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t xml:space="preserve">Equip. de Raios X - </t>
+          <t>Equip. ou Substancia</t>
         </is>
       </c>
       <c r="B236" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monoxido de Carbono </t>
+          <t xml:space="preserve">Aprision. Em, Sobre </t>
         </is>
       </c>
       <c r="B237" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elevador de Cacamba </t>
+          <t>Inalacao, Ingestao o</t>
         </is>
       </c>
       <c r="B238" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Inalacao de Substanc</t>
+          <t xml:space="preserve">Querosene           </t>
         </is>
       </c>
       <c r="B239" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Absorcao de Substanc</t>
+          <t>Dique, Barragem - Ed</t>
         </is>
       </c>
       <c r="B240" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Turbina             </t>
+          <t>Absorcao de Substanc</t>
         </is>
       </c>
       <c r="B241" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caixao Pneumatico - </t>
+          <t>Poluicao do Ar, Acao</t>
         </is>
       </c>
       <c r="B242" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Pele, Crina, Pelo, L</t>
+          <t>Ataque de Ser Vivo c</t>
         </is>
       </c>
       <c r="B243" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eletrica, Exposicao </t>
+          <t>Arquibancada, Estadi</t>
         </is>
       </c>
       <c r="B244" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Atrito ou Abrasao, N</t>
+          <t xml:space="preserve">Caixao Pneumatico - </t>
         </is>
       </c>
       <c r="B245" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Inalacao, Ingestao o</t>
+          <t>Composto Aromatico (</t>
         </is>
       </c>
       <c r="B246" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Oxidos de Nitrogenio</t>
+          <t xml:space="preserve">Produto de Petroleo </t>
         </is>
       </c>
       <c r="B247" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Composto Aromatico (</t>
+          <t>Embreagem de Friccao</t>
         </is>
       </c>
       <c r="B248" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Veiculo Funicular (T</t>
+          <t xml:space="preserve">Vibracao, Exposicao </t>
         </is>
       </c>
       <c r="B249" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Poluicao do Ar, Acao</t>
+          <t>Pena - Produto Anima</t>
         </is>
       </c>
       <c r="B250" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Pressao Ambiente Bai</t>
+          <t xml:space="preserve">Imersao             </t>
         </is>
       </c>
       <c r="B251" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vibracao, Exposicao </t>
+          <t>Aprision. Em, Sob ou</t>
         </is>
       </c>
       <c r="B252" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Pressao Ambiente Alt</t>
+          <t xml:space="preserve">Escafandro - Equip. </t>
         </is>
       </c>
       <c r="B253" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carvao              </t>
+          <t>Equip. de Mergulho -</t>
         </is>
       </c>
       <c r="B254" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Reator (Inclui Combu</t>
+          <t xml:space="preserve">Cianeto ou Composto </t>
         </is>
       </c>
       <c r="B255" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coque               </t>
+          <t xml:space="preserve">Eletrica, Exposicao </t>
         </is>
       </c>
       <c r="B256" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Querosene           </t>
+          <t>Pressao Ambiente Bai</t>
         </is>
       </c>
       <c r="B257" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Escafandro - Equip. </t>
+          <t xml:space="preserve">Turbina             </t>
         </is>
       </c>
       <c r="B258" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Equip. ou Substancia</t>
+          <t>Pressao Ambiente Alt</t>
         </is>
       </c>
       <c r="B259" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Aprision. Em, Sob ou</t>
+          <t>Oxidos de Nitrogenio</t>
         </is>
       </c>
       <c r="B260" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="inlineStr">
-        <is>
-          <t>Pena - Produto Anima</t>
-        </is>
-      </c>
-      <c r="B261" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t>Equip. de Mergulho -</t>
-        </is>
-      </c>
-      <c r="B262" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="inlineStr">
-        <is>
-          <t>Petroleo Bruto, Brut</t>
-        </is>
-      </c>
-      <c r="B263" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Composto de Fosforo </t>
-        </is>
-      </c>
-      <c r="B264" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="inlineStr">
-        <is>
-          <t>Radiacao nao Ionizan</t>
-        </is>
-      </c>
-      <c r="B265" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cianeto ou Composto </t>
-        </is>
-      </c>
-      <c r="B266" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Imersao             </t>
-        </is>
-      </c>
-      <c r="B267" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="inlineStr">
-        <is>
-          <t>Poluicao da Agua, Ac</t>
-        </is>
-      </c>
-      <c r="B268" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="inlineStr">
-        <is>
-          <t>Poluicao, Nic, Expos</t>
-        </is>
-      </c>
-      <c r="B269" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="inlineStr">
-        <is>
-          <t>Ingestao de Substanc</t>
-        </is>
-      </c>
-      <c r="B270" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="inlineStr">
-        <is>
-          <t>Temperatura Muito Ba</t>
-        </is>
-      </c>
-      <c r="B271" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Radiacao Ionizante, </t>
-        </is>
-      </c>
-      <c r="B272" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="inlineStr">
-        <is>
-          <t>Gas Encanado de Carv</t>
-        </is>
-      </c>
-      <c r="B273" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>